<commit_message>
fix(business): expand finance skill demo and preserve reading position
</commit_message>
<xml_diff>
--- a/public/samples/monthly-accounting.xlsx
+++ b/public/samples/monthly-accounting.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="売上データ" sheetId="1" r:id="Rfce7544f63534302"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入金明細" sheetId="2" r:id="R0af64b2fd494478d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="売上データ" sheetId="1" r:id="R512c534bc8644966"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入金明細" sheetId="2" r:id="R1764a3d3166d499d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -273,43 +273,37 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>取引先コード</x:v>
+        <x:v>取引先名</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>取引先名</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="str">
         <x:v>売上金額（円）</x:v>
       </x:c>
+      <x:c r="C1"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="1" t="str">
-        <x:v>C001</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="str">
         <x:v>山田商事</x:v>
       </x:c>
-      <x:c r="C2" s="4" t="n">
+      <x:c r="B2" s="4" t="n">
         <x:v>120000</x:v>
       </x:c>
+      <x:c r="C2"/>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>C002</x:v>
-      </x:c>
-      <x:c r="B3" s="5" t="str">
-        <x:v>田中工業（株）</x:v>
-      </x:c>
-      <x:c r="C3" s="6" t="n">
+        <x:v>田中工業</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="n">
         <x:v>230000</x:v>
       </x:c>
+      <x:c r="C3"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
@@ -325,43 +319,37 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>取引先コード</x:v>
+        <x:v>取引先名</x:v>
       </x:c>
       <x:c r="B1" s="3" t="str">
-        <x:v>取引先名</x:v>
-      </x:c>
-      <x:c r="C1" s="3" t="str">
         <x:v>入金額（円）</x:v>
       </x:c>
+      <x:c r="C1"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="1" t="str">
-        <x:v>C001</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="str">
-        <x:v>山田商事</x:v>
-      </x:c>
-      <x:c r="C2" s="4" t="n">
+        <x:v>山田商事 株式会社</x:v>
+      </x:c>
+      <x:c r="B2" s="4" t="n">
         <x:v>120000</x:v>
       </x:c>
+      <x:c r="C2"/>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="5" t="str">
-        <x:v>C002</x:v>
-      </x:c>
-      <x:c r="B3" s="5" t="str">
-        <x:v>田中工業株式会社</x:v>
-      </x:c>
-      <x:c r="C3" s="6" t="n">
+        <x:v>㈱田中工業</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="n">
         <x:v>200000</x:v>
       </x:c>
+      <x:c r="C3"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">

</xml_diff>